<commit_message>
Dashboard update 2026-08-11 21:32
</commit_message>
<xml_diff>
--- a/excel/Loanch Rima.xlsx
+++ b/excel/Loanch Rima.xlsx
@@ -5,25 +5,25 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.06.03\Loanch\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/69be8bcaca992739/Dokumentai/portfolio-analytics/portfolio-dashboard-clean/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D57DEA6-A7C9-4BC2-A6D6-C4CE53F612F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{4184CC5A-5D93-4FD8-A96D-732FB5F36FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{26591EF8-215E-47D1-93CB-094B11703178}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
     <sheet name="Pinigai" sheetId="15" r:id="rId2"/>
-    <sheet name="45b52ba0...0700af8e066e" sheetId="31" r:id="rId3"/>
-    <sheet name="4db6f5a8...8acf4fb9b90a" sheetId="30" r:id="rId4"/>
-    <sheet name="6836f159...155f27704bef" sheetId="29" r:id="rId5"/>
-    <sheet name="bab06fd6...b5601686ad35" sheetId="28" r:id="rId6"/>
-    <sheet name="6503e9b8...38a61e9781c1" sheetId="27" r:id="rId7"/>
-    <sheet name="edcaf7c8...13263f96f7ec" sheetId="26" r:id="rId8"/>
-    <sheet name="34060e5d...9d09fabf263e" sheetId="25" r:id="rId9"/>
-    <sheet name="8572f54e...85fb68b6201e" sheetId="24" r:id="rId10"/>
-    <sheet name="6a67a901...550919b8d681" sheetId="14" r:id="rId11"/>
+    <sheet name="eebd7526...eaf278164c4f" sheetId="31" r:id="rId3"/>
+    <sheet name="98b1dfe9...d5d30b41a3c0" sheetId="30" r:id="rId4"/>
+    <sheet name="63f224f9...dc9a9519a2fb" sheetId="29" r:id="rId5"/>
+    <sheet name="62dc7b87...555b6b58a73a" sheetId="28" r:id="rId6"/>
+    <sheet name="6a2ebaab...04ce88676cf8" sheetId="27" r:id="rId7"/>
+    <sheet name="6e656686...a6797d30436d-2" sheetId="26" r:id="rId8"/>
+    <sheet name="c78fc544...c7b919f73c9d" sheetId="25" r:id="rId9"/>
+    <sheet name="55bc6c86...98a4199721c7" sheetId="24" r:id="rId10"/>
+    <sheet name="6e656686...a6797d30436d-1" sheetId="14" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="55">
   <si>
     <t>Paskola</t>
   </si>
@@ -150,9 +150,6 @@
     <t>Nr.</t>
   </si>
   <si>
-    <t>6a67a901...550919b8d681</t>
-  </si>
-  <si>
     <t>Malaysia</t>
   </si>
   <si>
@@ -160,9 +157,6 @@
   </si>
   <si>
     <t>Short Term Loan</t>
-  </si>
-  <si>
-    <t>8572f54e...85fb68b6201e</t>
   </si>
   <si>
     <t>Liko, dienos</t>
@@ -183,31 +177,40 @@
     <t>Liko</t>
   </si>
   <si>
-    <t>34060e5d...9d09fabf263e</t>
-  </si>
-  <si>
-    <t>edcaf7c8...13263f96f7ec</t>
-  </si>
-  <si>
-    <t>6503e9b8...38a61e9781c1</t>
-  </si>
-  <si>
-    <t>bab06fd6...b5601686ad35</t>
-  </si>
-  <si>
     <t>Eur.</t>
-  </si>
-  <si>
-    <t>6836f159...155f27704bef</t>
-  </si>
-  <si>
-    <t>4db6f5a8...8acf4fb9b90a</t>
   </si>
   <si>
     <t xml:space="preserve">Premijos </t>
   </si>
   <si>
-    <t>45b52ba0...0700af8e066e</t>
+    <t>55bc6c86...98a4199721c7</t>
+  </si>
+  <si>
+    <t>c78fc544...c7b919f73c9d</t>
+  </si>
+  <si>
+    <t>6a2ebaab...04ce88676cf8</t>
+  </si>
+  <si>
+    <t>62dc7b87...555b6b58a73a</t>
+  </si>
+  <si>
+    <t>Installment Loan</t>
+  </si>
+  <si>
+    <t>63f224f9...dc9a9519a2fb</t>
+  </si>
+  <si>
+    <t>98b1dfe9...d5d30b41a3c0</t>
+  </si>
+  <si>
+    <t>eebd7526...eaf278164c4f</t>
+  </si>
+  <si>
+    <t>6e656686...a6797d30436d-1</t>
+  </si>
+  <si>
+    <t>6e656686...a6797d30436d-2</t>
   </si>
 </sst>
 </file>
@@ -1606,7 +1609,7 @@
         <v>33</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>3</v>
@@ -1633,10 +1636,10 @@
         <v>32</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M2" s="4" t="s">
         <v>0</v>
@@ -1655,7 +1658,7 @@
         <v>8</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="T2" s="4" t="s">
         <v>6</v>
@@ -1670,7 +1673,7 @@
         <v>24</v>
       </c>
       <c r="X2" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="Y2" s="4" t="s">
         <v>5</v>
@@ -1679,10 +1682,10 @@
         <v>26</v>
       </c>
       <c r="AA2" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="AC2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.25">
@@ -1690,69 +1693,69 @@
         <v>1</v>
       </c>
       <c r="B3" s="6">
-        <f>'8572f54e...85fb68b6201e'!B9</f>
-        <v>46140</v>
+        <f>'55bc6c86...98a4199721c7'!B9</f>
+        <v>46244</v>
       </c>
       <c r="C3" s="26" t="str">
-        <f>'6a67a901...550919b8d681'!B1</f>
-        <v>6a67a901...550919b8d681</v>
+        <f>'6e656686...a6797d30436d-1'!B1</f>
+        <v>6e656686...a6797d30436d-1</v>
       </c>
       <c r="D3" s="2" t="str">
-        <f>'6a67a901...550919b8d681'!B2</f>
+        <f>'6e656686...a6797d30436d-1'!B2</f>
         <v>Malaysia</v>
       </c>
       <c r="E3" s="2" t="str">
-        <f>'6a67a901...550919b8d681'!B3</f>
+        <f>'6e656686...a6797d30436d-1'!B3</f>
         <v>Tambadana</v>
       </c>
       <c r="F3" s="2" t="str">
-        <f>'6a67a901...550919b8d681'!B8</f>
-        <v>0 m. 1 mėn. 0 d.</v>
+        <f>'6e656686...a6797d30436d-1'!B8</f>
+        <v>0 m. 0 mėn. 30 d.</v>
       </c>
       <c r="G3" s="7">
-        <f>'6a67a901...550919b8d681'!B15</f>
+        <f>'6e656686...a6797d30436d-1'!B15</f>
         <v>0.13600000000000001</v>
       </c>
       <c r="H3" s="3">
-        <f>'6a67a901...550919b8d681'!B16</f>
+        <f>'6e656686...a6797d30436d-1'!B16</f>
         <v>10</v>
       </c>
       <c r="I3" s="6">
-        <f>'6a67a901...550919b8d681'!B11</f>
-        <v>46170</v>
-      </c>
-      <c r="J3" s="6">
-        <f>'6a67a901...550919b8d681'!O3</f>
-        <v>46154</v>
-      </c>
-      <c r="K3" s="19" t="str">
-        <f ca="1">'6a67a901...550919b8d681'!B12</f>
-        <v/>
+        <f>'6e656686...a6797d30436d-1'!B11</f>
+        <v>46274</v>
+      </c>
+      <c r="J3" s="6" t="str">
+        <f>'6e656686...a6797d30436d-1'!O3</f>
+        <v/>
+      </c>
+      <c r="K3" s="19">
+        <f ca="1">'6e656686...a6797d30436d-1'!B12</f>
+        <v>29</v>
       </c>
       <c r="L3" s="19" t="str">
-        <f ca="1">'6a67a901...550919b8d681'!P3</f>
+        <f ca="1">'6e656686...a6797d30436d-1'!P3</f>
         <v/>
       </c>
       <c r="M3" s="3">
-        <f>'6a67a901...550919b8d681'!K3</f>
-        <v>10</v>
+        <f>'6e656686...a6797d30436d-1'!K3</f>
+        <v>0</v>
       </c>
       <c r="N3" s="3">
-        <f>'6a67a901...550919b8d681'!L3</f>
-        <v>0.05</v>
+        <f>'6e656686...a6797d30436d-1'!L3</f>
+        <v>0</v>
       </c>
       <c r="O3" s="3">
-        <f>'6a67a901...550919b8d681'!M3</f>
+        <f>'6e656686...a6797d30436d-1'!M3</f>
         <v>0</v>
       </c>
       <c r="P3" s="10"/>
       <c r="Q3" s="29">
         <f>Pinigai!I2</f>
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="R3" s="29">
         <f>SUM(H3:H100)-U3</f>
-        <v>20.580000000000013</v>
+        <v>100</v>
       </c>
       <c r="S3" s="30">
         <f>Pinigai!H2</f>
@@ -1764,34 +1767,34 @@
       </c>
       <c r="U3" s="29">
         <f>SUM(M3:M100)</f>
-        <v>70.64</v>
+        <v>0</v>
       </c>
       <c r="V3" s="29">
         <f>SUM(N3:N100)-AA3</f>
-        <v>0.57999999999999996</v>
+        <v>0</v>
       </c>
       <c r="W3" s="29">
         <f>Q3+V3+S3</f>
-        <v>20.58</v>
+        <v>100</v>
       </c>
       <c r="X3" s="29">
         <f>W3-Q3</f>
-        <v>0.57999999999999829</v>
+        <v>0</v>
       </c>
       <c r="Y3" s="31">
         <f>(W3-Q3)/Q3</f>
-        <v>2.8999999999999915E-2</v>
+        <v>0</v>
       </c>
       <c r="Z3" s="31">
         <f ca="1">XIRR(Pinigai!K2:K200,Pinigai!A2:A200)</f>
-        <v>0.11481881737709046</v>
+        <v>2.9802322387695314E-9</v>
       </c>
       <c r="AA3" s="29">
         <f>SUM(O3:O100)</f>
         <v>0</v>
       </c>
       <c r="AC3" s="3" t="str">
-        <f ca="1">'6a67a901...550919b8d681'!Z3</f>
+        <f ca="1">'6e656686...a6797d30436d-1'!Z3</f>
         <v/>
       </c>
     </row>
@@ -1800,59 +1803,59 @@
         <v>2</v>
       </c>
       <c r="B4" s="6">
-        <f>'8572f54e...85fb68b6201e'!B9</f>
-        <v>46140</v>
+        <f>'55bc6c86...98a4199721c7'!B9</f>
+        <v>46244</v>
       </c>
       <c r="C4" s="26" t="str">
-        <f>'8572f54e...85fb68b6201e'!B1</f>
-        <v>8572f54e...85fb68b6201e</v>
+        <f>'55bc6c86...98a4199721c7'!B1</f>
+        <v>55bc6c86...98a4199721c7</v>
       </c>
       <c r="D4" s="2" t="str">
-        <f>'8572f54e...85fb68b6201e'!B2</f>
+        <f>'55bc6c86...98a4199721c7'!B2</f>
         <v>Malaysia</v>
       </c>
       <c r="E4" s="2" t="str">
-        <f>'8572f54e...85fb68b6201e'!B3</f>
+        <f>'55bc6c86...98a4199721c7'!B3</f>
         <v>Tambadana</v>
       </c>
       <c r="F4" s="2" t="str">
-        <f>'8572f54e...85fb68b6201e'!B8</f>
-        <v>0 m. 1 mėn. 0 d.</v>
+        <f>'55bc6c86...98a4199721c7'!B8</f>
+        <v>0 m. 0 mėn. 30 d.</v>
       </c>
       <c r="G4" s="7">
-        <f>'8572f54e...85fb68b6201e'!B15</f>
+        <f>'55bc6c86...98a4199721c7'!B15</f>
         <v>0.13600000000000001</v>
       </c>
       <c r="H4" s="3">
-        <f>'8572f54e...85fb68b6201e'!B16</f>
+        <f>'55bc6c86...98a4199721c7'!B16</f>
         <v>10</v>
       </c>
       <c r="I4" s="6">
-        <f>'8572f54e...85fb68b6201e'!B11</f>
-        <v>46170</v>
-      </c>
-      <c r="J4" s="6">
-        <f>'8572f54e...85fb68b6201e'!O3</f>
-        <v>46149</v>
-      </c>
-      <c r="K4" s="19" t="str">
-        <f ca="1">'8572f54e...85fb68b6201e'!B12</f>
-        <v/>
+        <f>'55bc6c86...98a4199721c7'!B11</f>
+        <v>46274</v>
+      </c>
+      <c r="J4" s="6" t="str">
+        <f>'55bc6c86...98a4199721c7'!O3</f>
+        <v/>
+      </c>
+      <c r="K4" s="19">
+        <f ca="1">'55bc6c86...98a4199721c7'!B12</f>
+        <v>29</v>
       </c>
       <c r="L4" s="19" t="str">
-        <f ca="1">'8572f54e...85fb68b6201e'!P3</f>
+        <f ca="1">'55bc6c86...98a4199721c7'!P3</f>
         <v/>
       </c>
       <c r="M4" s="3">
-        <f>'8572f54e...85fb68b6201e'!K3</f>
-        <v>10</v>
+        <f>'55bc6c86...98a4199721c7'!K3</f>
+        <v>0</v>
       </c>
       <c r="N4" s="3">
-        <f>'8572f54e...85fb68b6201e'!L3</f>
-        <v>0.03</v>
+        <f>'55bc6c86...98a4199721c7'!L3</f>
+        <v>0</v>
       </c>
       <c r="O4" s="3">
-        <f>'8572f54e...85fb68b6201e'!M3</f>
+        <f>'55bc6c86...98a4199721c7'!M3</f>
         <v>0</v>
       </c>
       <c r="P4" s="10"/>
@@ -1868,7 +1871,7 @@
       <c r="Z4" s="20"/>
       <c r="AA4" s="20"/>
       <c r="AC4" s="3" t="str">
-        <f ca="1">'8572f54e...85fb68b6201e'!Z3</f>
+        <f ca="1">'55bc6c86...98a4199721c7'!Z3</f>
         <v/>
       </c>
     </row>
@@ -1877,64 +1880,64 @@
         <v>3</v>
       </c>
       <c r="B5" s="6">
-        <f>'34060e5d...9d09fabf263e'!B9</f>
-        <v>46150</v>
+        <f>'c78fc544...c7b919f73c9d'!B9</f>
+        <v>46244</v>
       </c>
       <c r="C5" s="26" t="str">
-        <f>'34060e5d...9d09fabf263e'!B1</f>
-        <v>34060e5d...9d09fabf263e</v>
+        <f>'c78fc544...c7b919f73c9d'!B1</f>
+        <v>c78fc544...c7b919f73c9d</v>
       </c>
       <c r="D5" s="2" t="str">
-        <f>'34060e5d...9d09fabf263e'!B2</f>
+        <f>'c78fc544...c7b919f73c9d'!B2</f>
         <v>Malaysia</v>
       </c>
       <c r="E5" s="2" t="str">
-        <f>'34060e5d...9d09fabf263e'!B3</f>
+        <f>'c78fc544...c7b919f73c9d'!B3</f>
         <v>Tambadana</v>
       </c>
       <c r="F5" s="2" t="str">
-        <f>'34060e5d...9d09fabf263e'!B8</f>
-        <v>0 m. 1 mėn. 0 d.</v>
+        <f>'c78fc544...c7b919f73c9d'!B8</f>
+        <v>0 m. 3 mėn. 0 d.</v>
       </c>
       <c r="G5" s="7">
-        <f>'34060e5d...9d09fabf263e'!B15</f>
-        <v>0.13600000000000001</v>
+        <f>'c78fc544...c7b919f73c9d'!B15</f>
+        <v>0.159</v>
       </c>
       <c r="H5" s="3">
-        <f>'34060e5d...9d09fabf263e'!B16</f>
-        <v>10.029999999999999</v>
+        <f>'c78fc544...c7b919f73c9d'!B16</f>
+        <v>10</v>
       </c>
       <c r="I5" s="6">
-        <f>'34060e5d...9d09fabf263e'!B11</f>
-        <v>46181</v>
-      </c>
-      <c r="J5" s="6">
-        <f>'34060e5d...9d09fabf263e'!O3</f>
-        <v>46177</v>
-      </c>
-      <c r="K5" s="19" t="str">
-        <f ca="1">'34060e5d...9d09fabf263e'!B12</f>
-        <v/>
+        <f>'c78fc544...c7b919f73c9d'!B11</f>
+        <v>46336</v>
+      </c>
+      <c r="J5" s="6" t="str">
+        <f>'c78fc544...c7b919f73c9d'!O3</f>
+        <v/>
+      </c>
+      <c r="K5" s="19">
+        <f ca="1">'c78fc544...c7b919f73c9d'!B12</f>
+        <v>91</v>
       </c>
       <c r="L5" s="19" t="str">
-        <f ca="1">'34060e5d...9d09fabf263e'!P3</f>
+        <f ca="1">'c78fc544...c7b919f73c9d'!P3</f>
         <v/>
       </c>
       <c r="M5" s="3">
-        <f>'34060e5d...9d09fabf263e'!K3</f>
-        <v>10.029999999999999</v>
+        <f>'c78fc544...c7b919f73c9d'!K3</f>
+        <v>0</v>
       </c>
       <c r="N5" s="3">
-        <f>'34060e5d...9d09fabf263e'!L3</f>
-        <v>0.1</v>
+        <f>'c78fc544...c7b919f73c9d'!L3</f>
+        <v>0</v>
       </c>
       <c r="O5" s="3">
-        <f>'34060e5d...9d09fabf263e'!M3</f>
+        <f>'c78fc544...c7b919f73c9d'!M3</f>
         <v>0</v>
       </c>
       <c r="P5" s="10"/>
       <c r="AC5" s="3" t="str">
-        <f ca="1">'34060e5d...9d09fabf263e'!Z3</f>
+        <f ca="1">'c78fc544...c7b919f73c9d'!Z3</f>
         <v/>
       </c>
     </row>
@@ -1943,64 +1946,64 @@
         <v>4</v>
       </c>
       <c r="B6" s="6">
-        <f>'edcaf7c8...13263f96f7ec'!B9</f>
-        <v>46154</v>
+        <f>'6e656686...a6797d30436d-2'!B9</f>
+        <v>46244</v>
       </c>
       <c r="C6" s="26" t="str">
-        <f>'edcaf7c8...13263f96f7ec'!B1</f>
-        <v>edcaf7c8...13263f96f7ec</v>
+        <f>'6e656686...a6797d30436d-2'!B1</f>
+        <v>6e656686...a6797d30436d-2</v>
       </c>
       <c r="D6" s="2" t="str">
-        <f>'edcaf7c8...13263f96f7ec'!B2</f>
+        <f>'6e656686...a6797d30436d-2'!B2</f>
         <v>Malaysia</v>
       </c>
       <c r="E6" s="2" t="str">
-        <f>'edcaf7c8...13263f96f7ec'!B3</f>
+        <f>'6e656686...a6797d30436d-2'!B3</f>
         <v>Tambadana</v>
       </c>
       <c r="F6" s="2" t="str">
-        <f>'edcaf7c8...13263f96f7ec'!B8</f>
-        <v>0 m. 0 mėn. 1 d.</v>
+        <f>'6e656686...a6797d30436d-2'!B8</f>
+        <v>0 m. 0 mėn. 30 d.</v>
       </c>
       <c r="G6" s="7">
-        <f>'edcaf7c8...13263f96f7ec'!B15</f>
+        <f>'6e656686...a6797d30436d-2'!B15</f>
         <v>0.13600000000000001</v>
       </c>
       <c r="H6" s="3">
-        <f>'edcaf7c8...13263f96f7ec'!B16</f>
-        <v>10.050000000000001</v>
+        <f>'6e656686...a6797d30436d-2'!B16</f>
+        <v>10</v>
       </c>
       <c r="I6" s="6">
-        <f>'edcaf7c8...13263f96f7ec'!B11</f>
-        <v>46155</v>
-      </c>
-      <c r="J6" s="6">
-        <f>'edcaf7c8...13263f96f7ec'!O3</f>
-        <v>46185</v>
-      </c>
-      <c r="K6" s="19" t="str">
-        <f ca="1">'edcaf7c8...13263f96f7ec'!B12</f>
-        <v/>
+        <f>'6e656686...a6797d30436d-2'!B11</f>
+        <v>46274</v>
+      </c>
+      <c r="J6" s="6" t="str">
+        <f>'6e656686...a6797d30436d-2'!O3</f>
+        <v/>
+      </c>
+      <c r="K6" s="19">
+        <f ca="1">'6e656686...a6797d30436d-2'!B12</f>
+        <v>29</v>
       </c>
       <c r="L6" s="19" t="str">
-        <f ca="1">'edcaf7c8...13263f96f7ec'!P3</f>
+        <f ca="1">'6e656686...a6797d30436d-2'!P3</f>
         <v/>
       </c>
       <c r="M6" s="3">
-        <f>'edcaf7c8...13263f96f7ec'!K3</f>
-        <v>10.050000000000001</v>
+        <f>'6e656686...a6797d30436d-2'!K3</f>
+        <v>0</v>
       </c>
       <c r="N6" s="3">
-        <f>'edcaf7c8...13263f96f7ec'!L3</f>
-        <v>0.12</v>
+        <f>'6e656686...a6797d30436d-2'!L3</f>
+        <v>0</v>
       </c>
       <c r="O6" s="3">
-        <f>'edcaf7c8...13263f96f7ec'!M3</f>
+        <f>'6e656686...a6797d30436d-2'!M3</f>
         <v>0</v>
       </c>
       <c r="P6" s="10"/>
       <c r="AC6" s="3" t="str">
-        <f ca="1">'edcaf7c8...13263f96f7ec'!Z3</f>
+        <f ca="1">'6e656686...a6797d30436d-2'!Z3</f>
         <v/>
       </c>
     </row>
@@ -2009,64 +2012,64 @@
         <v>5</v>
       </c>
       <c r="B7" s="6">
-        <f>'6503e9b8...38a61e9781c1'!B9</f>
-        <v>46178</v>
+        <f>'6a2ebaab...04ce88676cf8'!B9</f>
+        <v>46244</v>
       </c>
       <c r="C7" s="26" t="str">
-        <f>'6503e9b8...38a61e9781c1'!B1</f>
-        <v>6503e9b8...38a61e9781c1</v>
+        <f>'6a2ebaab...04ce88676cf8'!B1</f>
+        <v>6a2ebaab...04ce88676cf8</v>
       </c>
       <c r="D7" s="2" t="str">
-        <f>'6503e9b8...38a61e9781c1'!B2</f>
+        <f>'6a2ebaab...04ce88676cf8'!B2</f>
         <v>Malaysia</v>
       </c>
       <c r="E7" s="2" t="str">
-        <f>'6503e9b8...38a61e9781c1'!B3</f>
+        <f>'6a2ebaab...04ce88676cf8'!B3</f>
         <v>Tambadana</v>
       </c>
       <c r="F7" s="2" t="str">
-        <f>'6503e9b8...38a61e9781c1'!B8</f>
-        <v>0 m. 1 mėn. 0 d.</v>
+        <f>'6a2ebaab...04ce88676cf8'!B8</f>
+        <v>0 m. 0 mėn. 30 d.</v>
       </c>
       <c r="G7" s="7">
-        <f>'6503e9b8...38a61e9781c1'!B15</f>
+        <f>'6a2ebaab...04ce88676cf8'!B15</f>
         <v>0.13600000000000001</v>
       </c>
       <c r="H7" s="3">
-        <f>'6503e9b8...38a61e9781c1'!B16</f>
-        <v>10.130000000000001</v>
+        <f>'6a2ebaab...04ce88676cf8'!B16</f>
+        <v>10</v>
       </c>
       <c r="I7" s="6">
-        <f>'6503e9b8...38a61e9781c1'!B11</f>
-        <v>46208</v>
-      </c>
-      <c r="J7" s="6">
-        <f>'6503e9b8...38a61e9781c1'!O3</f>
-        <v>46208</v>
-      </c>
-      <c r="K7" s="19" t="str">
-        <f ca="1">'6503e9b8...38a61e9781c1'!B12</f>
-        <v/>
+        <f>'6a2ebaab...04ce88676cf8'!B11</f>
+        <v>46274</v>
+      </c>
+      <c r="J7" s="6" t="str">
+        <f>'6a2ebaab...04ce88676cf8'!O3</f>
+        <v/>
+      </c>
+      <c r="K7" s="19">
+        <f ca="1">'6a2ebaab...04ce88676cf8'!B12</f>
+        <v>29</v>
       </c>
       <c r="L7" s="19" t="str">
-        <f ca="1">'6503e9b8...38a61e9781c1'!P3</f>
+        <f ca="1">'6a2ebaab...04ce88676cf8'!P3</f>
         <v/>
       </c>
       <c r="M7" s="3">
-        <f>'6503e9b8...38a61e9781c1'!K3</f>
-        <v>10.130000000000001</v>
+        <f>'6a2ebaab...04ce88676cf8'!K3</f>
+        <v>0</v>
       </c>
       <c r="N7" s="3">
-        <f>'6503e9b8...38a61e9781c1'!L3</f>
-        <v>0.11</v>
+        <f>'6a2ebaab...04ce88676cf8'!L3</f>
+        <v>0</v>
       </c>
       <c r="O7" s="3">
-        <f>'6503e9b8...38a61e9781c1'!M3</f>
+        <f>'6a2ebaab...04ce88676cf8'!M3</f>
         <v>0</v>
       </c>
       <c r="P7" s="10"/>
       <c r="AC7" s="3" t="str">
-        <f ca="1">'6503e9b8...38a61e9781c1'!Z3</f>
+        <f ca="1">'6a2ebaab...04ce88676cf8'!Z3</f>
         <v/>
       </c>
     </row>
@@ -2075,64 +2078,64 @@
         <v>6</v>
       </c>
       <c r="B8" s="6">
-        <f>'bab06fd6...b5601686ad35'!B9</f>
-        <v>46185</v>
+        <f>'62dc7b87...555b6b58a73a'!B9</f>
+        <v>46244</v>
       </c>
       <c r="C8" s="26" t="str">
-        <f>'bab06fd6...b5601686ad35'!B1</f>
-        <v>bab06fd6...b5601686ad35</v>
+        <f>'62dc7b87...555b6b58a73a'!B1</f>
+        <v>62dc7b87...555b6b58a73a</v>
       </c>
       <c r="D8" s="2" t="str">
-        <f>'bab06fd6...b5601686ad35'!B2</f>
+        <f>'62dc7b87...555b6b58a73a'!B2</f>
         <v>Malaysia</v>
       </c>
       <c r="E8" s="2" t="str">
-        <f>'bab06fd6...b5601686ad35'!B3</f>
+        <f>'62dc7b87...555b6b58a73a'!B3</f>
         <v>Tambadana</v>
       </c>
       <c r="F8" s="2" t="str">
-        <f>'bab06fd6...b5601686ad35'!B8</f>
-        <v>0 m. 1 mėn. 0 d.</v>
+        <f>'62dc7b87...555b6b58a73a'!B8</f>
+        <v>0 m. 3 mėn. 0 d.</v>
       </c>
       <c r="G8" s="7">
-        <f>'bab06fd6...b5601686ad35'!B15</f>
-        <v>0.13600000000000001</v>
+        <f>'62dc7b87...555b6b58a73a'!B15</f>
+        <v>0.159</v>
       </c>
       <c r="H8" s="3">
-        <f>'bab06fd6...b5601686ad35'!B16</f>
-        <v>10.17</v>
+        <f>'62dc7b87...555b6b58a73a'!B16</f>
+        <v>10</v>
       </c>
       <c r="I8" s="6">
-        <f>'bab06fd6...b5601686ad35'!B11</f>
-        <v>46215</v>
-      </c>
-      <c r="J8" s="6">
-        <f>'bab06fd6...b5601686ad35'!O3</f>
-        <v>46209</v>
-      </c>
-      <c r="K8" s="19" t="str">
-        <f ca="1">'bab06fd6...b5601686ad35'!B12</f>
-        <v/>
+        <f>'62dc7b87...555b6b58a73a'!B11</f>
+        <v>46336</v>
+      </c>
+      <c r="J8" s="6" t="str">
+        <f>'62dc7b87...555b6b58a73a'!O3</f>
+        <v/>
+      </c>
+      <c r="K8" s="19">
+        <f ca="1">'62dc7b87...555b6b58a73a'!B12</f>
+        <v>91</v>
       </c>
       <c r="L8" s="19" t="str">
-        <f ca="1">'bab06fd6...b5601686ad35'!P3</f>
+        <f ca="1">'62dc7b87...555b6b58a73a'!P3</f>
         <v/>
       </c>
       <c r="M8" s="3">
-        <f>'bab06fd6...b5601686ad35'!K3</f>
-        <v>10.17</v>
+        <f>'62dc7b87...555b6b58a73a'!K3</f>
+        <v>0</v>
       </c>
       <c r="N8" s="3">
-        <f>'bab06fd6...b5601686ad35'!L3</f>
-        <v>0.09</v>
+        <f>'62dc7b87...555b6b58a73a'!L3</f>
+        <v>0</v>
       </c>
       <c r="O8" s="3">
-        <f>'bab06fd6...b5601686ad35'!M3</f>
+        <f>'62dc7b87...555b6b58a73a'!M3</f>
         <v>0</v>
       </c>
       <c r="P8" s="10"/>
       <c r="AC8" s="3" t="str">
-        <f ca="1">'bab06fd6...b5601686ad35'!Z3</f>
+        <f ca="1">'62dc7b87...555b6b58a73a'!Z3</f>
         <v/>
       </c>
     </row>
@@ -2141,64 +2144,64 @@
         <v>7</v>
       </c>
       <c r="B9" s="6">
-        <f>'6836f159...155f27704bef'!B9</f>
-        <v>46208</v>
+        <f>'63f224f9...dc9a9519a2fb'!B9</f>
+        <v>46244</v>
       </c>
       <c r="C9" s="26" t="str">
-        <f>'6836f159...155f27704bef'!B1</f>
-        <v>6836f159...155f27704bef</v>
+        <f>'63f224f9...dc9a9519a2fb'!B1</f>
+        <v>63f224f9...dc9a9519a2fb</v>
       </c>
       <c r="D9" s="2" t="str">
-        <f>'6836f159...155f27704bef'!B2</f>
+        <f>'63f224f9...dc9a9519a2fb'!B2</f>
         <v>Malaysia</v>
       </c>
       <c r="E9" s="2" t="str">
-        <f>'6836f159...155f27704bef'!B3</f>
+        <f>'63f224f9...dc9a9519a2fb'!B3</f>
         <v>Tambadana</v>
       </c>
       <c r="F9" s="2" t="str">
-        <f>'6836f159...155f27704bef'!B8</f>
-        <v>0 m. 0 mėn. 30 d.</v>
+        <f>'63f224f9...dc9a9519a2fb'!B8</f>
+        <v>0 m. 3 mėn. 0 d.</v>
       </c>
       <c r="G9" s="7">
-        <f>'6836f159...155f27704bef'!B15</f>
-        <v>0.13600000000000001</v>
+        <f>'63f224f9...dc9a9519a2fb'!B15</f>
+        <v>0.159</v>
       </c>
       <c r="H9" s="3">
-        <f>'6836f159...155f27704bef'!B16</f>
-        <v>10.24</v>
+        <f>'63f224f9...dc9a9519a2fb'!B16</f>
+        <v>10</v>
       </c>
       <c r="I9" s="6">
-        <f>'6836f159...155f27704bef'!B11</f>
-        <v>46238</v>
+        <f>'63f224f9...dc9a9519a2fb'!B11</f>
+        <v>46336</v>
       </c>
       <c r="J9" s="6" t="str">
-        <f>'6836f159...155f27704bef'!O3</f>
+        <f>'63f224f9...dc9a9519a2fb'!O3</f>
         <v/>
       </c>
       <c r="K9" s="19">
-        <f ca="1">'6836f159...155f27704bef'!B12</f>
-        <v>3</v>
+        <f ca="1">'63f224f9...dc9a9519a2fb'!B12</f>
+        <v>91</v>
       </c>
       <c r="L9" s="19" t="str">
-        <f ca="1">'6836f159...155f27704bef'!P3</f>
+        <f ca="1">'63f224f9...dc9a9519a2fb'!P3</f>
         <v/>
       </c>
       <c r="M9" s="3">
-        <f>'6836f159...155f27704bef'!K3</f>
+        <f>'63f224f9...dc9a9519a2fb'!K3</f>
         <v>0</v>
       </c>
       <c r="N9" s="3">
-        <f>'6836f159...155f27704bef'!L3</f>
+        <f>'63f224f9...dc9a9519a2fb'!L3</f>
         <v>0</v>
       </c>
       <c r="O9" s="3">
-        <f>'6836f159...155f27704bef'!M3</f>
+        <f>'63f224f9...dc9a9519a2fb'!M3</f>
         <v>0</v>
       </c>
       <c r="P9" s="10"/>
       <c r="AC9" s="3" t="str">
-        <f ca="1">'6836f159...155f27704bef'!Z3</f>
+        <f ca="1">'63f224f9...dc9a9519a2fb'!Z3</f>
         <v/>
       </c>
     </row>
@@ -2207,64 +2210,64 @@
         <v>8</v>
       </c>
       <c r="B10" s="6">
-        <f>'4db6f5a8...8acf4fb9b90a'!B9</f>
-        <v>46209</v>
+        <f>'98b1dfe9...d5d30b41a3c0'!B9</f>
+        <v>46244</v>
       </c>
       <c r="C10" s="26" t="str">
-        <f>'4db6f5a8...8acf4fb9b90a'!B1</f>
-        <v>4db6f5a8...8acf4fb9b90a</v>
+        <f>'98b1dfe9...d5d30b41a3c0'!B1</f>
+        <v>98b1dfe9...d5d30b41a3c0</v>
       </c>
       <c r="D10" s="2" t="str">
-        <f>'4db6f5a8...8acf4fb9b90a'!B2</f>
+        <f>'98b1dfe9...d5d30b41a3c0'!B2</f>
         <v>Malaysia</v>
       </c>
       <c r="E10" s="2" t="str">
-        <f>'4db6f5a8...8acf4fb9b90a'!B3</f>
+        <f>'98b1dfe9...d5d30b41a3c0'!B3</f>
         <v>Tambadana</v>
       </c>
       <c r="F10" s="2" t="str">
-        <f>'4db6f5a8...8acf4fb9b90a'!B8</f>
-        <v>0 m. 0 mėn. 30 d.</v>
+        <f>'98b1dfe9...d5d30b41a3c0'!B8</f>
+        <v>0 m. 3 mėn. 0 d.</v>
       </c>
       <c r="G10" s="7">
-        <f>'4db6f5a8...8acf4fb9b90a'!B15</f>
-        <v>0.13600000000000001</v>
+        <f>'98b1dfe9...d5d30b41a3c0'!B15</f>
+        <v>0.159</v>
       </c>
       <c r="H10" s="3">
-        <f>'4db6f5a8...8acf4fb9b90a'!B16</f>
-        <v>10.26</v>
+        <f>'98b1dfe9...d5d30b41a3c0'!B16</f>
+        <v>15</v>
       </c>
       <c r="I10" s="6">
-        <f>'4db6f5a8...8acf4fb9b90a'!B11</f>
-        <v>46239</v>
-      </c>
-      <c r="J10" s="6">
-        <f>'4db6f5a8...8acf4fb9b90a'!O3</f>
-        <v>46231</v>
-      </c>
-      <c r="K10" s="19" t="str">
-        <f ca="1">'4db6f5a8...8acf4fb9b90a'!B12</f>
-        <v/>
+        <f>'98b1dfe9...d5d30b41a3c0'!B11</f>
+        <v>46336</v>
+      </c>
+      <c r="J10" s="6" t="str">
+        <f>'98b1dfe9...d5d30b41a3c0'!O3</f>
+        <v/>
+      </c>
+      <c r="K10" s="19">
+        <f ca="1">'98b1dfe9...d5d30b41a3c0'!B12</f>
+        <v>91</v>
       </c>
       <c r="L10" s="19" t="str">
-        <f ca="1">'4db6f5a8...8acf4fb9b90a'!P3</f>
+        <f ca="1">'98b1dfe9...d5d30b41a3c0'!P3</f>
         <v/>
       </c>
       <c r="M10" s="3">
-        <f>'4db6f5a8...8acf4fb9b90a'!K3</f>
-        <v>10.26</v>
+        <f>'98b1dfe9...d5d30b41a3c0'!K3</f>
+        <v>0</v>
       </c>
       <c r="N10" s="3">
-        <f>'4db6f5a8...8acf4fb9b90a'!L3</f>
-        <v>0.08</v>
+        <f>'98b1dfe9...d5d30b41a3c0'!L3</f>
+        <v>0</v>
       </c>
       <c r="O10" s="3">
-        <f>'4db6f5a8...8acf4fb9b90a'!M3</f>
+        <f>'98b1dfe9...d5d30b41a3c0'!M3</f>
         <v>0</v>
       </c>
       <c r="P10" s="10"/>
       <c r="AC10" s="3" t="str">
-        <f ca="1">'4db6f5a8...8acf4fb9b90a'!Z3</f>
+        <f ca="1">'98b1dfe9...d5d30b41a3c0'!Z3</f>
         <v/>
       </c>
     </row>
@@ -2273,64 +2276,64 @@
         <v>9</v>
       </c>
       <c r="B11" s="6">
-        <f>'45b52ba0...0700af8e066e'!B9</f>
-        <v>46231</v>
+        <f>'eebd7526...eaf278164c4f'!B9</f>
+        <v>46244</v>
       </c>
       <c r="C11" s="26" t="str">
-        <f>'45b52ba0...0700af8e066e'!B1</f>
-        <v>45b52ba0...0700af8e066e</v>
+        <f>'eebd7526...eaf278164c4f'!B1</f>
+        <v>eebd7526...eaf278164c4f</v>
       </c>
       <c r="D11" s="2" t="str">
-        <f>'45b52ba0...0700af8e066e'!B2</f>
+        <f>'eebd7526...eaf278164c4f'!B2</f>
         <v>Malaysia</v>
       </c>
       <c r="E11" s="2" t="str">
-        <f>'45b52ba0...0700af8e066e'!B3</f>
+        <f>'eebd7526...eaf278164c4f'!B3</f>
         <v>Tambadana</v>
       </c>
       <c r="F11" s="2" t="str">
-        <f>'45b52ba0...0700af8e066e'!B8</f>
-        <v>0 m. 0 mėn. 30 d.</v>
+        <f>'eebd7526...eaf278164c4f'!B8</f>
+        <v>0 m. 3 mėn. 0 d.</v>
       </c>
       <c r="G11" s="7">
-        <f>'45b52ba0...0700af8e066e'!B15</f>
-        <v>0.13600000000000001</v>
+        <f>'eebd7526...eaf278164c4f'!B15</f>
+        <v>0.159</v>
       </c>
       <c r="H11" s="3">
-        <f>'45b52ba0...0700af8e066e'!B16</f>
-        <v>10.34</v>
+        <f>'eebd7526...eaf278164c4f'!B16</f>
+        <v>15</v>
       </c>
       <c r="I11" s="6">
-        <f>'45b52ba0...0700af8e066e'!B11</f>
-        <v>46261</v>
+        <f>'eebd7526...eaf278164c4f'!B11</f>
+        <v>46336</v>
       </c>
       <c r="J11" s="6" t="str">
-        <f>'45b52ba0...0700af8e066e'!O3</f>
+        <f>'eebd7526...eaf278164c4f'!O3</f>
         <v/>
       </c>
       <c r="K11" s="19">
-        <f ca="1">'45b52ba0...0700af8e066e'!B12</f>
-        <v>26</v>
+        <f ca="1">'eebd7526...eaf278164c4f'!B12</f>
+        <v>91</v>
       </c>
       <c r="L11" s="19" t="str">
-        <f ca="1">'45b52ba0...0700af8e066e'!P3</f>
+        <f ca="1">'eebd7526...eaf278164c4f'!P3</f>
         <v/>
       </c>
       <c r="M11" s="3">
-        <f>'45b52ba0...0700af8e066e'!K3</f>
+        <f>'eebd7526...eaf278164c4f'!K3</f>
         <v>0</v>
       </c>
       <c r="N11" s="3">
-        <f>'45b52ba0...0700af8e066e'!L3</f>
+        <f>'eebd7526...eaf278164c4f'!L3</f>
         <v>0</v>
       </c>
       <c r="O11" s="3">
-        <f>'45b52ba0...0700af8e066e'!M3</f>
+        <f>'eebd7526...eaf278164c4f'!M3</f>
         <v>0</v>
       </c>
       <c r="P11" s="10"/>
       <c r="AC11" s="3" t="str">
-        <f ca="1">'45b52ba0...0700af8e066e'!Z3</f>
+        <f ca="1">'eebd7526...eaf278164c4f'!Z3</f>
         <v/>
       </c>
     </row>
@@ -2650,15 +2653,15 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="C3" location="'6a67a901...550919b8d681'!A1" display="'6a67a901...550919b8d681'!A1" xr:uid="{87C3E6BC-C2D4-4CD6-83E2-4126641D3546}"/>
-    <hyperlink ref="C4" location="'8572f54e...85fb68b6201e'!A1" display="'8572f54e...85fb68b6201e'!A1" xr:uid="{E1A2E8FA-E90A-432F-B098-8C25480A0509}"/>
-    <hyperlink ref="C5" location="'34060e5d...9d09fabf263e'!A1" display="'34060e5d...9d09fabf263e'!A1" xr:uid="{DD06AB51-16D7-406E-BEFF-B6F40935BA74}"/>
-    <hyperlink ref="C6" location="edcaf7c8...13263f96f7ec!A1" display="edcaf7c8...13263f96f7ec!A1" xr:uid="{E78838E4-E5C7-443E-82BB-4777748DBDD8}"/>
-    <hyperlink ref="C7" location="'edcaf7c8...13263f96f7ec (2)'!A1" display="'edcaf7c8...13263f96f7ec (2)'!A1" xr:uid="{A45ECDA9-CD3D-488B-8BD0-974ED148F5E4}"/>
-    <hyperlink ref="C8" location="bab06fd6...b5601686ad35!A1" display="bab06fd6...b5601686ad35!A1" xr:uid="{CF3F48D9-3FC3-49AA-8DA2-BFA6E5A240F1}"/>
-    <hyperlink ref="C9" location="'6836f159...155f27704bef'!A1" display="'6836f159...155f27704bef'!A1" xr:uid="{6FBE713B-C5C1-4487-AEB0-76FB8384D359}"/>
-    <hyperlink ref="C10" location="'4db6f5a8...8acf4fb9b90a'!A1" display="'4db6f5a8...8acf4fb9b90a'!A1" xr:uid="{51C54BD2-6758-450A-BD35-5AEE8C98C71A}"/>
-    <hyperlink ref="C11" location="'45b52ba0...0700af8e066e'!A1" display="'45b52ba0...0700af8e066e'!A1" xr:uid="{99FD08BF-C515-4DD4-9F3D-763A30898E51}"/>
+    <hyperlink ref="C3" location="'6e656686...a6797d30436d-1'!A1" display="'6e656686...a6797d30436d-1'!A1" xr:uid="{87C3E6BC-C2D4-4CD6-83E2-4126641D3546}"/>
+    <hyperlink ref="C4" location="'55bc6c86...98a4199721c7'!A1" display="'55bc6c86...98a4199721c7'!A1" xr:uid="{E1A2E8FA-E90A-432F-B098-8C25480A0509}"/>
+    <hyperlink ref="C5" location="'c78fc544...c7b919f73c9d'!A1" display="'c78fc544...c7b919f73c9d'!A1" xr:uid="{DD06AB51-16D7-406E-BEFF-B6F40935BA74}"/>
+    <hyperlink ref="C6" location="'6e656686...a6797d30436d-2'!A1" display="'6e656686...a6797d30436d-2'!A1" xr:uid="{E78838E4-E5C7-443E-82BB-4777748DBDD8}"/>
+    <hyperlink ref="C7" location="'6a2ebaab...04ce88676cf8'!A1" display="'6a2ebaab...04ce88676cf8'!A1" xr:uid="{A45ECDA9-CD3D-488B-8BD0-974ED148F5E4}"/>
+    <hyperlink ref="C8" location="'62dc7b87...555b6b58a73a'!A1" display="'62dc7b87...555b6b58a73a'!A1" xr:uid="{CF3F48D9-3FC3-49AA-8DA2-BFA6E5A240F1}"/>
+    <hyperlink ref="C9" location="'63f224f9...dc9a9519a2fb'!A1" display="'63f224f9...dc9a9519a2fb'!A1" xr:uid="{6FBE713B-C5C1-4487-AEB0-76FB8384D359}"/>
+    <hyperlink ref="C10" location="'98b1dfe9...d5d30b41a3c0'!A1" display="'98b1dfe9...d5d30b41a3c0'!A1" xr:uid="{51C54BD2-6758-450A-BD35-5AEE8C98C71A}"/>
+    <hyperlink ref="C11" location="eebd7526...eaf278164c4f!A1" display="eebd7526...eaf278164c4f!A1" xr:uid="{99FD08BF-C515-4DD4-9F3D-763A30898E51}"/>
   </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="50" orientation="landscape" r:id="rId1"/>
@@ -2667,9 +2670,6 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{583E60DD-D268-4B5D-B986-F933A571227C}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2693,7 +2693,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D1" s="32" t="s">
         <v>2</v>
@@ -2724,7 +2724,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>31</v>
@@ -2733,7 +2733,7 @@
         <v>32</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>12</v>
@@ -2761,10 +2761,10 @@
         <v>2</v>
       </c>
       <c r="P2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="X2" s="12" t="s">
         <v>2</v>
@@ -2773,7 +2773,7 @@
         <v>28</v>
       </c>
       <c r="Z2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
@@ -2781,60 +2781,52 @@
         <v>18</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D3" s="11">
-        <v>46170</v>
-      </c>
-      <c r="E3" s="6">
-        <v>46149</v>
-      </c>
-      <c r="F3" s="19">
+        <v>46274</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="19" t="str">
         <f>IF(E3&gt;0,E3-D3,"")</f>
-        <v>-21</v>
-      </c>
-      <c r="G3" s="3">
-        <v>10</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0.03</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="14"/>
       <c r="K3" s="3">
         <f>G53</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
         <v>0</v>
       </c>
-      <c r="N3" s="7">
+      <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
-        <v>0.12917190194129949</v>
-      </c>
-      <c r="O3" s="6">
+        <v/>
+      </c>
+      <c r="O3" s="6" t="str">
         <f>IF(B16=K3,MAX(E:E),"")</f>
-        <v>46149</v>
+        <v/>
       </c>
       <c r="P3" s="2" t="str">
         <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
         <v/>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="2" t="str">
         <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
-        <v>-21</v>
+        <v/>
       </c>
       <c r="T3" s="13"/>
       <c r="X3" s="6">
         <f>B9</f>
-        <v>46140</v>
+        <v>46244</v>
       </c>
       <c r="Y3" s="3">
         <f>B16*-1</f>
@@ -2850,7 +2842,7 @@
         <v>19</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="6"/>
@@ -2864,11 +2856,11 @@
       <c r="J4" s="10"/>
       <c r="X4" s="6">
         <f>E3</f>
-        <v>46149</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="3">
         <f>G3+H3-I3</f>
-        <v>10.029999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
@@ -2943,7 +2935,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
-        <v>0 m. 1 mėn. 0 d.</v>
+        <v>0 m. 0 mėn. 30 d.</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="6"/>
@@ -2969,7 +2961,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6">
-        <v>46140</v>
+        <v>46244</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="6"/>
@@ -2995,7 +2987,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="6">
-        <v>46140</v>
+        <v>46244</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="6"/>
@@ -3021,7 +3013,7 @@
         <v>30</v>
       </c>
       <c r="B11" s="6">
-        <v>46170</v>
+        <v>46274</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="6"/>
@@ -3044,11 +3036,11 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="19" t="str">
+        <v>37</v>
+      </c>
+      <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v/>
+        <v>29</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -3149,7 +3141,7 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B16" s="3">
         <v>10</v>
@@ -3909,11 +3901,11 @@
       <c r="F53" s="3"/>
       <c r="G53" s="3">
         <f>SUM(G3:G52)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
@@ -3953,9 +3945,6 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3979,7 +3968,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="D1" s="32" t="s">
         <v>2</v>
@@ -4010,7 +3999,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>31</v>
@@ -4019,7 +4008,7 @@
         <v>32</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>12</v>
@@ -4047,10 +4036,10 @@
         <v>2</v>
       </c>
       <c r="P2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="X2" s="12" t="s">
         <v>2</v>
@@ -4059,7 +4048,7 @@
         <v>28</v>
       </c>
       <c r="Z2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
@@ -4067,60 +4056,52 @@
         <v>18</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D3" s="11">
-        <v>46170</v>
-      </c>
-      <c r="E3" s="6">
-        <v>46154</v>
-      </c>
-      <c r="F3" s="19">
+        <v>46274</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="19" t="str">
         <f>IF(E3&gt;0,E3-D3,"")</f>
-        <v>-16</v>
-      </c>
-      <c r="G3" s="3">
-        <v>10</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0.05</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="14"/>
       <c r="K3" s="3">
         <f>G53</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
         <v>0</v>
       </c>
-      <c r="N3" s="7">
+      <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
-        <v>0.13886520266532895</v>
-      </c>
-      <c r="O3" s="6">
+        <v/>
+      </c>
+      <c r="O3" s="6" t="str">
         <f>IF(B16=K3,MAX(E:E),"")</f>
-        <v>46154</v>
+        <v/>
       </c>
       <c r="P3" s="2" t="str">
         <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
         <v/>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="2" t="str">
         <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
-        <v>-16</v>
+        <v/>
       </c>
       <c r="T3" s="13"/>
       <c r="X3" s="6">
         <f>B9</f>
-        <v>46140</v>
+        <v>46244</v>
       </c>
       <c r="Y3" s="3">
         <f>B16*-1</f>
@@ -4136,7 +4117,7 @@
         <v>19</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="6"/>
@@ -4150,11 +4131,11 @@
       <c r="J4" s="10"/>
       <c r="X4" s="6">
         <f>E3</f>
-        <v>46154</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="3">
         <f>G3+H3-I3</f>
-        <v>10.050000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
@@ -4229,7 +4210,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
-        <v>0 m. 1 mėn. 0 d.</v>
+        <v>0 m. 0 mėn. 30 d.</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="6"/>
@@ -4255,7 +4236,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6">
-        <v>46140</v>
+        <v>46244</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="6"/>
@@ -4281,7 +4262,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="6">
-        <v>46140</v>
+        <v>46244</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="6"/>
@@ -4307,7 +4288,7 @@
         <v>30</v>
       </c>
       <c r="B11" s="6">
-        <v>46170</v>
+        <v>46274</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="6"/>
@@ -4330,11 +4311,11 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="19" t="str">
+        <v>37</v>
+      </c>
+      <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v/>
+        <v>29</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -4435,7 +4416,7 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B16" s="3">
         <v>10</v>
@@ -5194,11 +5175,11 @@
       <c r="F53" s="3"/>
       <c r="G53" s="3">
         <f>SUM(G3:G52)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
@@ -5279,10 +5260,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="6">
-        <v>46139</v>
+        <v>46242</v>
       </c>
       <c r="B2" s="3">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="C2" s="3">
         <v>0</v>
@@ -5292,7 +5273,7 @@
       </c>
       <c r="F2" s="3">
         <f>SUM(B2:B35)</f>
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="G2" s="3">
         <f>SUM(C2:C35)</f>
@@ -5304,11 +5285,11 @@
       </c>
       <c r="I2" s="3">
         <f>F2-G2</f>
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="K2" s="3">
         <f>B2*-1</f>
-        <v>-20</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -6693,14 +6674,14 @@
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200" s="15">
         <f ca="1">TODAY()</f>
-        <v>46235</v>
+        <v>46245</v>
       </c>
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
       <c r="D200" s="1"/>
       <c r="K200" s="3">
         <f>Overview!W3</f>
-        <v>20.58</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -6733,7 +6714,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D1" s="32" t="s">
         <v>2</v>
@@ -6764,7 +6745,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>31</v>
@@ -6773,7 +6754,7 @@
         <v>32</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>12</v>
@@ -6801,10 +6782,10 @@
         <v>2</v>
       </c>
       <c r="P2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="X2" s="12" t="s">
         <v>2</v>
@@ -6813,7 +6794,7 @@
         <v>28</v>
       </c>
       <c r="Z2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
@@ -6821,10 +6802,10 @@
         <v>18</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D3" s="11">
-        <v>46238</v>
+        <v>46275</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="19" t="str">
@@ -6866,11 +6847,11 @@
       <c r="T3" s="13"/>
       <c r="X3" s="6">
         <f>B9</f>
-        <v>46231</v>
+        <v>46244</v>
       </c>
       <c r="Y3" s="3">
         <f>B16*-1</f>
-        <v>-10.34</v>
+        <v>-15</v>
       </c>
       <c r="Z3" s="2" t="str">
         <f ca="1">IF(AND(TODAY()&gt;B11, K3&lt;&gt;B16), "+", "")</f>
@@ -6882,9 +6863,11 @@
         <v>19</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="11"/>
+        <v>49</v>
+      </c>
+      <c r="D4" s="11">
+        <v>46305</v>
+      </c>
       <c r="E4" s="6"/>
       <c r="F4" s="19" t="str">
         <f>IF(E4&gt;0,E4-D4,"")</f>
@@ -6906,7 +6889,9 @@
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="6"/>
-      <c r="D5" s="11"/>
+      <c r="D5" s="11">
+        <v>46336</v>
+      </c>
       <c r="E5" s="6"/>
       <c r="F5" s="19" t="str">
         <f t="shared" ref="F5:F52" si="0">IF(E5&gt;0,E5-D5,"")</f>
@@ -6975,7 +6960,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
-        <v>0 m. 0 mėn. 30 d.</v>
+        <v>0 m. 3 mėn. 0 d.</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="6"/>
@@ -7001,7 +6986,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6">
-        <v>46231</v>
+        <v>46244</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="6"/>
@@ -7027,7 +7012,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="6">
-        <v>46231</v>
+        <v>46244</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="6"/>
@@ -7053,7 +7038,7 @@
         <v>30</v>
       </c>
       <c r="B11" s="6">
-        <v>46261</v>
+        <v>46336</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="6"/>
@@ -7076,11 +7061,11 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>26</v>
+        <v>91</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -7151,7 +7136,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="7">
-        <v>0.13600000000000001</v>
+        <v>0.159</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="6"/>
@@ -7181,10 +7166,10 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B16" s="3">
-        <v>10.34</v>
+        <v>15</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="6"/>
@@ -7985,9 +7970,6 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{355B2BCE-B3A8-4634-BB20-53D0C8F481D1}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8042,7 +8024,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>31</v>
@@ -8051,7 +8033,7 @@
         <v>32</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>12</v>
@@ -8079,10 +8061,10 @@
         <v>2</v>
       </c>
       <c r="P2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="X2" s="12" t="s">
         <v>2</v>
@@ -8091,7 +8073,7 @@
         <v>28</v>
       </c>
       <c r="Z2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
@@ -8099,64 +8081,56 @@
         <v>18</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D3" s="11">
-        <v>46239</v>
-      </c>
-      <c r="E3" s="6">
-        <v>46231</v>
-      </c>
-      <c r="F3" s="19">
+        <v>46275</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="19" t="str">
         <f>IF(E3&gt;0,E3-D3,"")</f>
-        <v>-8</v>
-      </c>
-      <c r="G3" s="3">
-        <v>10.26</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0.08</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="14"/>
       <c r="K3" s="3">
         <f>G53</f>
-        <v>10.26</v>
+        <v>0</v>
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
         <v>0</v>
       </c>
-      <c r="N3" s="7">
+      <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
-        <v>0.13753321766853335</v>
-      </c>
-      <c r="O3" s="6">
+        <v/>
+      </c>
+      <c r="O3" s="6" t="str">
         <f>IF(B16=K3,MAX(E:E),"")</f>
-        <v>46231</v>
+        <v/>
       </c>
       <c r="P3" s="2" t="str">
         <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
         <v/>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="2" t="str">
         <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
-        <v>-8</v>
+        <v/>
       </c>
       <c r="T3" s="13"/>
       <c r="X3" s="6">
         <f>B9</f>
-        <v>46209</v>
+        <v>46244</v>
       </c>
       <c r="Y3" s="3">
         <f>B16*-1</f>
-        <v>-10.26</v>
+        <v>-15</v>
       </c>
       <c r="Z3" s="2" t="str">
         <f ca="1">IF(AND(TODAY()&gt;B11, K3&lt;&gt;B16), "+", "")</f>
@@ -8168,9 +8142,11 @@
         <v>19</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="11"/>
+        <v>49</v>
+      </c>
+      <c r="D4" s="11">
+        <v>46305</v>
+      </c>
       <c r="E4" s="6"/>
       <c r="F4" s="19" t="str">
         <f>IF(E4&gt;0,E4-D4,"")</f>
@@ -8182,17 +8158,19 @@
       <c r="J4" s="10"/>
       <c r="X4" s="6">
         <f>E3</f>
-        <v>46231</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="3">
         <f>G3+H3-I3</f>
-        <v>10.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="6"/>
-      <c r="D5" s="11"/>
+      <c r="D5" s="11">
+        <v>46336</v>
+      </c>
       <c r="E5" s="6"/>
       <c r="F5" s="19" t="str">
         <f t="shared" ref="F5:F52" si="0">IF(E5&gt;0,E5-D5,"")</f>
@@ -8261,7 +8239,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
-        <v>0 m. 0 mėn. 30 d.</v>
+        <v>0 m. 3 mėn. 0 d.</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="6"/>
@@ -8287,7 +8265,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6">
-        <v>46209</v>
+        <v>46244</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="6"/>
@@ -8313,7 +8291,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="6">
-        <v>46209</v>
+        <v>46244</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="6"/>
@@ -8339,7 +8317,7 @@
         <v>30</v>
       </c>
       <c r="B11" s="6">
-        <v>46239</v>
+        <v>46336</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="6"/>
@@ -8362,11 +8340,11 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="19" t="str">
+        <v>37</v>
+      </c>
+      <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v/>
+        <v>91</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -8437,7 +8415,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="7">
-        <v>0.13600000000000001</v>
+        <v>0.159</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="6"/>
@@ -8467,10 +8445,10 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B16" s="3">
-        <v>10.26</v>
+        <v>15</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="6"/>
@@ -9227,11 +9205,11 @@
       <c r="F53" s="3"/>
       <c r="G53" s="3">
         <f>SUM(G3:G52)</f>
-        <v>10.26</v>
+        <v>0</v>
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
@@ -9325,7 +9303,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>31</v>
@@ -9334,7 +9312,7 @@
         <v>32</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>12</v>
@@ -9362,10 +9340,10 @@
         <v>2</v>
       </c>
       <c r="P2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="X2" s="12" t="s">
         <v>2</v>
@@ -9374,7 +9352,7 @@
         <v>28</v>
       </c>
       <c r="Z2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
@@ -9382,10 +9360,10 @@
         <v>18</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D3" s="11">
-        <v>46238</v>
+        <v>46275</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="19" t="str">
@@ -9427,11 +9405,11 @@
       <c r="T3" s="13"/>
       <c r="X3" s="6">
         <f>B9</f>
-        <v>46208</v>
+        <v>46244</v>
       </c>
       <c r="Y3" s="3">
         <f>B16*-1</f>
-        <v>-10.24</v>
+        <v>-10</v>
       </c>
       <c r="Z3" s="2" t="str">
         <f ca="1">IF(AND(TODAY()&gt;B11, K3&lt;&gt;B16), "+", "")</f>
@@ -9443,9 +9421,11 @@
         <v>19</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="11"/>
+        <v>49</v>
+      </c>
+      <c r="D4" s="11">
+        <v>46305</v>
+      </c>
       <c r="E4" s="6"/>
       <c r="F4" s="19" t="str">
         <f>IF(E4&gt;0,E4-D4,"")</f>
@@ -9467,7 +9447,9 @@
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="6"/>
-      <c r="D5" s="11"/>
+      <c r="D5" s="11">
+        <v>46336</v>
+      </c>
       <c r="E5" s="6"/>
       <c r="F5" s="19" t="str">
         <f t="shared" ref="F5:F52" si="0">IF(E5&gt;0,E5-D5,"")</f>
@@ -9536,7 +9518,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
-        <v>0 m. 0 mėn. 30 d.</v>
+        <v>0 m. 3 mėn. 0 d.</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="6"/>
@@ -9562,7 +9544,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6">
-        <v>46208</v>
+        <v>46244</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="6"/>
@@ -9588,7 +9570,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="6">
-        <v>46208</v>
+        <v>46244</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="6"/>
@@ -9614,7 +9596,7 @@
         <v>30</v>
       </c>
       <c r="B11" s="6">
-        <v>46238</v>
+        <v>46336</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="6"/>
@@ -9637,11 +9619,11 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>3</v>
+        <v>91</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -9712,7 +9694,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="7">
-        <v>0.13600000000000001</v>
+        <v>0.159</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="6"/>
@@ -9742,10 +9724,10 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B16" s="3">
-        <v>10.24</v>
+        <v>10</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="6"/>
@@ -10546,9 +10528,6 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05E38648-85FB-451A-8C48-F23050BE99C9}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -10603,7 +10582,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>31</v>
@@ -10612,7 +10591,7 @@
         <v>32</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>12</v>
@@ -10640,10 +10619,10 @@
         <v>2</v>
       </c>
       <c r="P2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="X2" s="12" t="s">
         <v>2</v>
@@ -10652,7 +10631,7 @@
         <v>28</v>
       </c>
       <c r="Z2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
@@ -10660,64 +10639,56 @@
         <v>18</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D3" s="11">
-        <v>46215</v>
-      </c>
-      <c r="E3" s="6">
-        <v>46209</v>
-      </c>
-      <c r="F3" s="19">
+        <v>46275</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="19" t="str">
         <f>IF(E3&gt;0,E3-D3,"")</f>
-        <v>-6</v>
-      </c>
-      <c r="G3" s="3">
-        <v>10.17</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0.09</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="14"/>
       <c r="K3" s="3">
         <f>G53</f>
-        <v>10.17</v>
+        <v>0</v>
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
         <v>0</v>
       </c>
-      <c r="N3" s="7">
+      <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
-        <v>0.14338709712028502</v>
-      </c>
-      <c r="O3" s="6">
+        <v/>
+      </c>
+      <c r="O3" s="6" t="str">
         <f>IF(B16=K3,MAX(E:E),"")</f>
-        <v>46209</v>
+        <v/>
       </c>
       <c r="P3" s="2" t="str">
         <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
         <v/>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="2" t="str">
         <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
-        <v>-6</v>
+        <v/>
       </c>
       <c r="T3" s="13"/>
       <c r="X3" s="6">
         <f>B9</f>
-        <v>46185</v>
+        <v>46244</v>
       </c>
       <c r="Y3" s="3">
         <f>B16*-1</f>
-        <v>-10.17</v>
+        <v>-10</v>
       </c>
       <c r="Z3" s="2" t="str">
         <f ca="1">IF(AND(TODAY()&gt;B11, K3&lt;&gt;B16), "+", "")</f>
@@ -10729,9 +10700,11 @@
         <v>19</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="11"/>
+        <v>49</v>
+      </c>
+      <c r="D4" s="11">
+        <v>46305</v>
+      </c>
       <c r="E4" s="6"/>
       <c r="F4" s="19" t="str">
         <f>IF(E4&gt;0,E4-D4,"")</f>
@@ -10743,17 +10716,19 @@
       <c r="J4" s="10"/>
       <c r="X4" s="6">
         <f>E3</f>
-        <v>46209</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="3">
         <f>G3+H3-I3</f>
-        <v>10.26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="6"/>
-      <c r="D5" s="11"/>
+      <c r="D5" s="11">
+        <v>46336</v>
+      </c>
       <c r="E5" s="6"/>
       <c r="F5" s="19" t="str">
         <f t="shared" ref="F5:F52" si="0">IF(E5&gt;0,E5-D5,"")</f>
@@ -10822,7 +10797,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
-        <v>0 m. 1 mėn. 0 d.</v>
+        <v>0 m. 3 mėn. 0 d.</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="6"/>
@@ -10848,7 +10823,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6">
-        <v>46185</v>
+        <v>46244</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="6"/>
@@ -10874,7 +10849,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="6">
-        <v>46185</v>
+        <v>46244</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="6"/>
@@ -10900,7 +10875,7 @@
         <v>30</v>
       </c>
       <c r="B11" s="6">
-        <v>46215</v>
+        <v>46336</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="6"/>
@@ -10923,11 +10898,11 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="19" t="str">
+        <v>37</v>
+      </c>
+      <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v/>
+        <v>91</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -10998,7 +10973,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="7">
-        <v>0.13600000000000001</v>
+        <v>0.159</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="6"/>
@@ -11028,10 +11003,10 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B16" s="3">
-        <v>10.17</v>
+        <v>10</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="6"/>
@@ -11788,11 +11763,11 @@
       <c r="F53" s="3"/>
       <c r="G53" s="3">
         <f>SUM(G3:G52)</f>
-        <v>10.17</v>
+        <v>0</v>
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
@@ -11832,9 +11807,6 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CFD3710-89A2-4F7D-A324-B3CED3BB72D8}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -11889,7 +11861,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>31</v>
@@ -11898,7 +11870,7 @@
         <v>32</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>12</v>
@@ -11926,10 +11898,10 @@
         <v>2</v>
       </c>
       <c r="P2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="X2" s="12" t="s">
         <v>2</v>
@@ -11938,7 +11910,7 @@
         <v>28</v>
       </c>
       <c r="Z2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
@@ -11946,64 +11918,56 @@
         <v>18</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D3" s="11">
-        <v>46208</v>
-      </c>
-      <c r="E3" s="6">
-        <v>46208</v>
-      </c>
-      <c r="F3" s="19">
+        <v>46274</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="19" t="str">
         <f>IF(E3&gt;0,E3-D3,"")</f>
-        <v>0</v>
-      </c>
-      <c r="G3" s="3">
-        <v>10.130000000000001</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0.11</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="14"/>
       <c r="K3" s="3">
         <f>G53</f>
-        <v>10.130000000000001</v>
+        <v>0</v>
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
         <v>0</v>
       </c>
-      <c r="N3" s="7">
+      <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
-        <v>0.14042803645133972</v>
-      </c>
-      <c r="O3" s="6">
+        <v/>
+      </c>
+      <c r="O3" s="6" t="str">
         <f>IF(B16=K3,MAX(E:E),"")</f>
-        <v>46208</v>
+        <v/>
       </c>
       <c r="P3" s="2" t="str">
         <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
         <v/>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="2" t="str">
         <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="T3" s="13"/>
       <c r="X3" s="6">
         <f>B9</f>
-        <v>46178</v>
+        <v>46244</v>
       </c>
       <c r="Y3" s="3">
         <f>B16*-1</f>
-        <v>-10.130000000000001</v>
+        <v>-10</v>
       </c>
       <c r="Z3" s="2" t="str">
         <f ca="1">IF(AND(TODAY()&gt;B11, K3&lt;&gt;B16), "+", "")</f>
@@ -12015,7 +11979,7 @@
         <v>19</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="6"/>
@@ -12029,11 +11993,11 @@
       <c r="J4" s="10"/>
       <c r="X4" s="6">
         <f>E3</f>
-        <v>46208</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="3">
         <f>G3+H3-I3</f>
-        <v>10.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
@@ -12108,7 +12072,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
-        <v>0 m. 1 mėn. 0 d.</v>
+        <v>0 m. 0 mėn. 30 d.</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="6"/>
@@ -12134,7 +12098,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6">
-        <v>46178</v>
+        <v>46244</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="6"/>
@@ -12160,7 +12124,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="6">
-        <v>46178</v>
+        <v>46244</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="6"/>
@@ -12186,7 +12150,7 @@
         <v>30</v>
       </c>
       <c r="B11" s="6">
-        <v>46208</v>
+        <v>46274</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="6"/>
@@ -12209,11 +12173,11 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="19" t="str">
+        <v>37</v>
+      </c>
+      <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v/>
+        <v>29</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -12314,10 +12278,10 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B16" s="3">
-        <v>10.130000000000001</v>
+        <v>10</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="6"/>
@@ -13074,11 +13038,11 @@
       <c r="F53" s="3"/>
       <c r="G53" s="3">
         <f>SUM(G3:G52)</f>
-        <v>10.130000000000001</v>
+        <v>0</v>
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
@@ -13118,9 +13082,6 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{894C5DD5-26F0-4BD8-A02A-9EA73D3EF2C5}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -13144,7 +13105,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="D1" s="32" t="s">
         <v>2</v>
@@ -13175,7 +13136,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>31</v>
@@ -13184,7 +13145,7 @@
         <v>32</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>12</v>
@@ -13212,10 +13173,10 @@
         <v>2</v>
       </c>
       <c r="P2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="X2" s="12" t="s">
         <v>2</v>
@@ -13224,7 +13185,7 @@
         <v>28</v>
       </c>
       <c r="Z2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
@@ -13232,64 +13193,56 @@
         <v>18</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D3" s="11">
-        <v>46155</v>
-      </c>
-      <c r="E3" s="6">
-        <v>46185</v>
-      </c>
-      <c r="F3" s="19">
+        <v>46274</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="19" t="str">
         <f>IF(E3&gt;0,E3-D3,"")</f>
-        <v>30</v>
-      </c>
-      <c r="G3" s="3">
-        <v>10.050000000000001</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0.12</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="14"/>
       <c r="K3" s="3">
         <f>G53</f>
-        <v>10.050000000000001</v>
+        <v>0</v>
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
         <v>0</v>
       </c>
-      <c r="N3" s="7">
+      <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
-        <v>0.14999164938926698</v>
-      </c>
-      <c r="O3" s="6">
+        <v/>
+      </c>
+      <c r="O3" s="6" t="str">
         <f>IF(B16=K3,MAX(E:E),"")</f>
-        <v>46185</v>
+        <v/>
       </c>
       <c r="P3" s="2" t="str">
         <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
         <v/>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="2" t="str">
         <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
-        <v>30</v>
+        <v/>
       </c>
       <c r="T3" s="13"/>
       <c r="X3" s="6">
         <f>B9</f>
-        <v>46154</v>
+        <v>46244</v>
       </c>
       <c r="Y3" s="3">
         <f>B16*-1</f>
-        <v>-10.050000000000001</v>
+        <v>-10</v>
       </c>
       <c r="Z3" s="2" t="str">
         <f ca="1">IF(AND(TODAY()&gt;B11, K3&lt;&gt;B16), "+", "")</f>
@@ -13301,7 +13254,7 @@
         <v>19</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="6"/>
@@ -13315,11 +13268,11 @@
       <c r="J4" s="10"/>
       <c r="X4" s="6">
         <f>E3</f>
-        <v>46185</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="3">
         <f>G3+H3-I3</f>
-        <v>10.17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
@@ -13394,7 +13347,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
-        <v>0 m. 0 mėn. 1 d.</v>
+        <v>0 m. 0 mėn. 30 d.</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="6"/>
@@ -13420,7 +13373,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6">
-        <v>46154</v>
+        <v>46244</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="6"/>
@@ -13446,7 +13399,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="6">
-        <v>46124</v>
+        <v>46244</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="6"/>
@@ -13472,7 +13425,7 @@
         <v>30</v>
       </c>
       <c r="B11" s="6">
-        <v>46155</v>
+        <v>46274</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="6"/>
@@ -13495,11 +13448,11 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="19" t="str">
+        <v>37</v>
+      </c>
+      <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v/>
+        <v>29</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -13600,10 +13553,10 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B16" s="3">
-        <v>10.050000000000001</v>
+        <v>10</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="6"/>
@@ -14360,11 +14313,11 @@
       <c r="F53" s="3"/>
       <c r="G53" s="3">
         <f>SUM(G3:G52)</f>
-        <v>10.050000000000001</v>
+        <v>0</v>
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
@@ -14404,9 +14357,6 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D73BEB5-FF23-4AB2-910E-BFC1E1552858}">
-  <sheetPr>
-    <tabColor rgb="FF92D050"/>
-  </sheetPr>
   <dimension ref="A1:Z53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -14430,7 +14380,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D1" s="32" t="s">
         <v>2</v>
@@ -14461,7 +14411,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>31</v>
@@ -14470,7 +14420,7 @@
         <v>32</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>12</v>
@@ -14498,10 +14448,10 @@
         <v>2</v>
       </c>
       <c r="P2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="X2" s="12" t="s">
         <v>2</v>
@@ -14510,7 +14460,7 @@
         <v>28</v>
       </c>
       <c r="Z2" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
@@ -14518,64 +14468,56 @@
         <v>18</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D3" s="11">
-        <v>46181</v>
-      </c>
-      <c r="E3" s="6">
-        <v>46177</v>
-      </c>
-      <c r="F3" s="19">
+        <v>46275</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="19" t="str">
         <f>IF(E3&gt;0,E3-D3,"")</f>
-        <v>-4</v>
-      </c>
-      <c r="G3" s="3">
-        <v>10.029999999999999</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0.1</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="14"/>
       <c r="K3" s="3">
         <f>G53</f>
-        <v>10.029999999999999</v>
+        <v>0</v>
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
         <v>0</v>
       </c>
-      <c r="N3" s="7">
+      <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
-        <v>0.1435224711894989</v>
-      </c>
-      <c r="O3" s="6">
+        <v/>
+      </c>
+      <c r="O3" s="6" t="str">
         <f>IF(B16=K3,MAX(E:E),"")</f>
-        <v>46177</v>
+        <v/>
       </c>
       <c r="P3" s="2" t="str">
         <f ca="1">IF(Z3="+",TODAY()-B11,"")</f>
         <v/>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="2" t="str">
         <f>IF(B16=K3,MAX(E:E)-B11,"")</f>
-        <v>-4</v>
+        <v/>
       </c>
       <c r="T3" s="13"/>
       <c r="X3" s="6">
         <f>B9</f>
-        <v>46150</v>
+        <v>46244</v>
       </c>
       <c r="Y3" s="3">
         <f>B16*-1</f>
-        <v>-10.029999999999999</v>
+        <v>-10</v>
       </c>
       <c r="Z3" s="2" t="str">
         <f ca="1">IF(AND(TODAY()&gt;B11, K3&lt;&gt;B16), "+", "")</f>
@@ -14587,9 +14529,11 @@
         <v>19</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="11"/>
+        <v>49</v>
+      </c>
+      <c r="D4" s="11">
+        <v>46305</v>
+      </c>
       <c r="E4" s="6"/>
       <c r="F4" s="19" t="str">
         <f>IF(E4&gt;0,E4-D4,"")</f>
@@ -14601,17 +14545,19 @@
       <c r="J4" s="10"/>
       <c r="X4" s="6">
         <f>E3</f>
-        <v>46177</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="3">
         <f>G3+H3-I3</f>
-        <v>10.129999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="6"/>
-      <c r="D5" s="11"/>
+      <c r="D5" s="11">
+        <v>46336</v>
+      </c>
       <c r="E5" s="6"/>
       <c r="F5" s="19" t="str">
         <f t="shared" ref="F5:F52" si="0">IF(E5&gt;0,E5-D5,"")</f>
@@ -14680,7 +14626,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f>DATEDIF(B9,B11,"y") &amp; " m. " &amp; DATEDIF(B9,B11,"ym") &amp; " mėn. " &amp; DATEDIF(B9,B11,"md") &amp; " d."</f>
-        <v>0 m. 1 mėn. 0 d.</v>
+        <v>0 m. 3 mėn. 0 d.</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="6"/>
@@ -14706,7 +14652,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6">
-        <v>46150</v>
+        <v>46244</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="6"/>
@@ -14732,7 +14678,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="6">
-        <v>46150</v>
+        <v>46244</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="6"/>
@@ -14758,7 +14704,7 @@
         <v>30</v>
       </c>
       <c r="B11" s="6">
-        <v>46181</v>
+        <v>46336</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="6"/>
@@ -14781,11 +14727,11 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="19" t="str">
+        <v>37</v>
+      </c>
+      <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v/>
+        <v>91</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -14856,7 +14802,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="7">
-        <v>0.13600000000000001</v>
+        <v>0.159</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="6"/>
@@ -14886,10 +14832,10 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B16" s="3">
-        <v>10.029999999999999</v>
+        <v>10</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="6"/>
@@ -15646,11 +15592,11 @@
       <c r="F53" s="3"/>
       <c r="G53" s="3">
         <f>SUM(G3:G52)</f>
-        <v>10.029999999999999</v>
+        <v>0</v>
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>

</xml_diff>